<commit_message>
case studies with 10 dd
</commit_message>
<xml_diff>
--- a/case_studies/base_case_10_dd/2020/technologies.xlsx
+++ b/case_studies/base_case_10_dd/2020/technologies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\base_case_5_dd\2020\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F6D653-8C50-4C49-9B7B-31FC524023C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="3" r:id="rId1"/>
@@ -470,9 +470,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A32646D9-68BB-474D-B725-BABE5F54D2FA}">
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -567,7 +567,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -662,7 +662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -757,7 +757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -852,7 +852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -947,7 +947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1240,9 +1240,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B7B1BB4-9645-4A08-BE86-AFBC7A2F79A5}">
   <dimension ref="A1:Z8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1890,9 +1890,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD6448D7-10EE-4973-BCA6-F7E0B963E195}">
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2082,7 +2082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -2462,7 +2462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2557,7 +2557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>25</v>
       </c>

</xml_diff>